<commit_message>
Added Exercise 4C .xlsx
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_more_GTrends.xlsx
+++ b/week-01/Ex4A_more_GTrends.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tihitinazergaw\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2AA1CE4-85F8-4BE3-AE60-94149F2E7D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0306ADF7-B6D5-4F46-A650-2BEEC5B5744B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D55DA867-9CC0-4163-85D6-76E0045C0D68}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet1!$A$1:$D$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>